<commit_message>
Update offer management and trial mngt
</commit_message>
<xml_diff>
--- a/The_Prompt_Studio_Production_Checklist.xlsx
+++ b/The_Prompt_Studio_Production_Checklist.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mathieuthiao-layel/Documents/promptcraft/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05CE0B7B-AAA4-4242-824C-09A592C000F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE82FE3B-3543-5D48-8054-F90EACACA45A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="780" windowWidth="34200" windowHeight="21460" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="68800" windowHeight="28800" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Checklist Production" sheetId="1" r:id="rId1"/>
@@ -821,22 +821,9 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -875,6 +862,19 @@
     <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1145,2051 +1145,2051 @@
   <dimension ref="A1:G126"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="5" customWidth="1"/>
-    <col min="2" max="2" width="8" customWidth="1"/>
-    <col min="3" max="3" width="50" customWidth="1"/>
-    <col min="4" max="4" width="35" customWidth="1"/>
-    <col min="5" max="5" width="20" customWidth="1"/>
-    <col min="6" max="6" width="15" customWidth="1"/>
-    <col min="7" max="7" width="20" customWidth="1"/>
+    <col min="1" max="1" width="30.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="53.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="69.83203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.1640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="49.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
+      <c r="F1" s="26"/>
+      <c r="G1" s="26"/>
     </row>
     <row r="2" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="4" t="s">
+      <c r="A2" s="27" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
+      <c r="B2" s="27"/>
+      <c r="C2" s="27"/>
+      <c r="D2" s="27"/>
+      <c r="E2" s="27"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
     </row>
     <row r="3" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="3" t="s">
+      <c r="A3" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="3"/>
-      <c r="C3" s="6" t="str">
+      <c r="B3" s="28"/>
+      <c r="C3" s="3" t="str">
         <f>CONCATENATE(COUNTIF(A5:A200,"✅")," / ",COUNTA(C5:C200)," tâches complétées (",ROUND(COUNTIF(A5:A200,"✅")/MAX(COUNTA(C5:C200),1)*100,0),"%)")</f>
-        <v>23 / 69 tâches complétées (33%)</v>
-      </c>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
-      <c r="G3" s="7"/>
+        <v>25 / 69 tâches complétées (36%)</v>
+      </c>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
     </row>
     <row r="4" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="8" t="s">
+      <c r="B4" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="C4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="D4" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="E4" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="F4" s="8" t="s">
+      <c r="F4" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="G4" s="8" t="s">
+      <c r="G4" s="5" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="24" t="s">
         <v>10</v>
       </c>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
+      <c r="B5" s="24"/>
+      <c r="C5" s="24"/>
+      <c r="D5" s="24"/>
+      <c r="E5" s="24"/>
+      <c r="F5" s="24"/>
+      <c r="G5" s="24"/>
     </row>
     <row r="6" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="11" t="s">
+      <c r="B6" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="C6" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="D6" s="13" t="s">
+      <c r="D6" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="E6" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F6" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G6" s="13"/>
+      <c r="E6" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F6" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G6" s="8"/>
     </row>
     <row r="7" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="10" t="s">
+      <c r="A7" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="11" t="s">
+      <c r="B7" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="C7" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="D7" s="13" t="s">
+      <c r="D7" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="E7" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F7" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G7" s="13"/>
+      <c r="E7" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F7" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G7" s="8"/>
     </row>
     <row r="8" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="10" t="s">
+      <c r="A8" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="11" t="s">
+      <c r="B8" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="12" t="s">
+      <c r="C8" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="13" t="s">
+      <c r="D8" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="E8" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F8" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G8" s="13"/>
+      <c r="E8" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F8" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G8" s="8"/>
     </row>
     <row r="9" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="10" t="s">
+      <c r="A9" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="B9" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="12" t="s">
+      <c r="C9" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="D9" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="E9" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F9" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G9" s="13"/>
+      <c r="E9" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F9" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G9" s="8"/>
     </row>
     <row r="10" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="2" t="s">
+      <c r="A10" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
+      <c r="B10" s="24"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
+      <c r="G10" s="24"/>
     </row>
     <row r="11" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="10" t="s">
+      <c r="A11" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B11" s="11" t="s">
+      <c r="B11" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C11" s="12" t="s">
+      <c r="C11" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="D11" s="13" t="s">
+      <c r="D11" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="E11" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F11" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G11" s="13"/>
+      <c r="E11" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F11" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G11" s="8"/>
     </row>
     <row r="12" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="10" t="s">
+      <c r="A12" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B12" s="11" t="s">
+      <c r="B12" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C12" s="12" t="s">
+      <c r="C12" s="7" t="s">
         <v>26</v>
       </c>
-      <c r="D12" s="13" t="s">
+      <c r="D12" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="E12" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F12" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G12" s="13"/>
+      <c r="E12" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F12" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G12" s="8"/>
     </row>
     <row r="13" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="10" t="s">
+      <c r="A13" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="B13" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C13" s="12" t="s">
+      <c r="C13" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="D13" s="13" t="s">
+      <c r="D13" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="E13" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F13" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G13" s="13"/>
+      <c r="E13" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F13" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G13" s="8"/>
     </row>
     <row r="14" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="10" t="s">
+      <c r="A14" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B14" s="11" t="s">
+      <c r="B14" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C14" s="12" t="s">
+      <c r="C14" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="D14" s="13" t="s">
+      <c r="D14" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="E14" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F14" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G14" s="13"/>
+      <c r="E14" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F14" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G14" s="8"/>
     </row>
     <row r="15" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="10" t="s">
+      <c r="A15" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B15" s="11" t="s">
+      <c r="B15" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C15" s="12" t="s">
+      <c r="C15" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="D15" s="13" t="s">
+      <c r="D15" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="E15" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F15" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G15" s="13"/>
+      <c r="E15" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F15" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G15" s="8"/>
     </row>
     <row r="16" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="10" t="s">
+      <c r="A16" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B16" s="11" t="s">
+      <c r="B16" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C16" s="12" t="s">
+      <c r="C16" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="D16" s="13" t="s">
+      <c r="D16" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="E16" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F16" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G16" s="13"/>
+      <c r="E16" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F16" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G16" s="8"/>
     </row>
     <row r="17" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="10" t="s">
+      <c r="A17" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B17" s="11" t="s">
+      <c r="B17" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C17" s="12" t="s">
+      <c r="C17" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="D17" s="15" t="s">
+      <c r="D17" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="E17" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F17" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G17" s="13"/>
+      <c r="E17" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F17" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G17" s="8"/>
     </row>
     <row r="18" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="2" t="s">
+      <c r="A18" s="24" t="s">
         <v>38</v>
       </c>
-      <c r="B18" s="2"/>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
+      <c r="B18" s="24"/>
+      <c r="C18" s="24"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="24"/>
+      <c r="F18" s="24"/>
+      <c r="G18" s="24"/>
     </row>
     <row r="19" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="10" t="s">
+      <c r="A19" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B19" s="11" t="s">
+      <c r="B19" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C19" s="12" t="s">
+      <c r="C19" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="D19" s="13" t="s">
+      <c r="D19" s="8" t="s">
         <v>40</v>
       </c>
-      <c r="E19" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F19" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G19" s="13"/>
+      <c r="E19" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F19" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G19" s="8"/>
     </row>
     <row r="20" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="10" t="s">
+      <c r="A20" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B20" s="11" t="s">
+      <c r="B20" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C20" s="12" t="s">
+      <c r="C20" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="D20" s="13" t="s">
+      <c r="D20" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="E20" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F20" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G20" s="13"/>
+      <c r="E20" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F20" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G20" s="8"/>
     </row>
     <row r="21" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="10" t="s">
+      <c r="A21" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B21" s="11" t="s">
+      <c r="B21" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C21" s="12" t="s">
+      <c r="C21" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="D21" s="13" t="s">
+      <c r="D21" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="E21" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F21" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G21" s="13"/>
+      <c r="E21" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F21" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G21" s="8"/>
     </row>
     <row r="22" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="10" t="s">
+      <c r="A22" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B22" s="11" t="s">
+      <c r="B22" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C22" s="12" t="s">
+      <c r="C22" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="D22" s="13" t="s">
+      <c r="D22" s="8" t="s">
         <v>46</v>
       </c>
-      <c r="E22" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F22" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G22" s="13"/>
+      <c r="E22" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F22" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G22" s="8"/>
     </row>
     <row r="23" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="10" t="s">
+      <c r="A23" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="B23" s="11" t="s">
+      <c r="B23" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C23" s="12" t="s">
+      <c r="C23" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="D23" s="13" t="s">
+      <c r="D23" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="E23" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F23" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G23" s="13"/>
+      <c r="E23" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F23" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G23" s="8"/>
     </row>
     <row r="24" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="2" t="s">
+      <c r="A24" s="24" t="s">
         <v>50</v>
       </c>
-      <c r="B24" s="2"/>
-      <c r="C24" s="2"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-      <c r="F24" s="2"/>
-      <c r="G24" s="2"/>
+      <c r="B24" s="24"/>
+      <c r="C24" s="24"/>
+      <c r="D24" s="24"/>
+      <c r="E24" s="24"/>
+      <c r="F24" s="24"/>
+      <c r="G24" s="24"/>
     </row>
     <row r="25" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="10" t="s">
+      <c r="A25" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B25" s="11" t="s">
+      <c r="B25" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C25" s="12" t="s">
+      <c r="C25" s="7" t="s">
         <v>51</v>
       </c>
-      <c r="D25" s="13" t="s">
+      <c r="D25" s="8" t="s">
         <v>52</v>
       </c>
-      <c r="E25" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F25" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G25" s="13"/>
+      <c r="E25" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F25" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G25" s="8"/>
     </row>
     <row r="26" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="10" t="s">
+      <c r="A26" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B26" s="11" t="s">
+      <c r="B26" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C26" s="12" t="s">
+      <c r="C26" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="D26" s="13" t="s">
+      <c r="D26" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="E26" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F26" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G26" s="13"/>
+      <c r="E26" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F26" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G26" s="8"/>
     </row>
     <row r="27" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="10" t="s">
+      <c r="A27" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="B27" s="11" t="s">
+      <c r="B27" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C27" s="12" t="s">
+      <c r="C27" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="D27" s="13" t="s">
+      <c r="D27" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="E27" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F27" s="14" t="s">
+      <c r="E27" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F27" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G27" s="13" t="s">
+      <c r="G27" s="8" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="32.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="10" t="s">
+      <c r="A28" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B28" s="11" t="s">
+      <c r="B28" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C28" s="12" t="s">
+      <c r="C28" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="D28" s="13" t="s">
+      <c r="D28" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="E28" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F28" s="14" t="s">
+      <c r="E28" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F28" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G28" s="13" t="s">
+      <c r="G28" s="8" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="29" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B29" s="11" t="s">
+      <c r="A29" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B29" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="C29" s="12" t="s">
+      <c r="C29" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="D29" s="16" t="s">
+      <c r="D29" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="E29" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F29" s="14" t="s">
+      <c r="E29" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F29" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="G29" s="13" t="s">
+      <c r="G29" s="8" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="17" t="s">
-        <v>59</v>
-      </c>
-      <c r="B30" s="18" t="s">
+      <c r="A30" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="B30" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="C30" s="17" t="s">
+      <c r="C30" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="D30" s="18" t="s">
+      <c r="D30" s="13" t="s">
         <v>69</v>
       </c>
-      <c r="E30" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="F30" s="19" t="s">
+      <c r="E30" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="F30" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="G30" s="18"/>
+      <c r="G30" s="13"/>
     </row>
     <row r="31" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="17" t="s">
-        <v>59</v>
-      </c>
-      <c r="B31" s="18" t="s">
+      <c r="A31" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="B31" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="C31" s="17" t="s">
+      <c r="C31" s="12" t="s">
         <v>70</v>
       </c>
-      <c r="D31" s="18" t="s">
+      <c r="D31" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="E31" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="F31" s="19" t="s">
+      <c r="E31" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="F31" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="G31" s="18" t="s">
+      <c r="G31" s="13" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="17" t="s">
-        <v>59</v>
-      </c>
-      <c r="B32" s="18" t="s">
+      <c r="A32" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="B32" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="C32" s="17" t="s">
+      <c r="C32" s="12" t="s">
         <v>73</v>
       </c>
-      <c r="D32" s="18" t="s">
+      <c r="D32" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="E32" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="F32" s="19" t="s">
+      <c r="E32" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="F32" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="G32" s="18" t="s">
+      <c r="G32" s="13" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="17" t="s">
-        <v>59</v>
-      </c>
-      <c r="B33" s="18" t="s">
+      <c r="A33" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="B33" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="C33" s="17" t="s">
+      <c r="C33" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="D33" s="18" t="s">
+      <c r="D33" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="E33" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="F33" s="19" t="s">
+      <c r="E33" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="F33" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="G33" s="18"/>
+      <c r="G33" s="13"/>
     </row>
     <row r="34" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="17" t="s">
-        <v>59</v>
-      </c>
-      <c r="B34" s="18" t="s">
+      <c r="A34" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="B34" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="C34" s="17" t="s">
+      <c r="C34" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="D34" s="18" t="s">
+      <c r="D34" s="13" t="s">
         <v>79</v>
       </c>
-      <c r="E34" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="F34" s="19" t="s">
+      <c r="E34" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="F34" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="G34" s="18" t="s">
+      <c r="G34" s="13" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="35" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="9" t="s">
+      <c r="A35" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="B35" s="20"/>
-      <c r="C35" s="20"/>
-      <c r="D35" s="20"/>
-      <c r="E35" s="20"/>
-      <c r="F35" s="20"/>
-      <c r="G35" s="20"/>
+      <c r="B35" s="15"/>
+      <c r="C35" s="15"/>
+      <c r="D35" s="15"/>
+      <c r="E35" s="15"/>
+      <c r="F35" s="15"/>
+      <c r="G35" s="15"/>
     </row>
     <row r="36" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A36" s="10" t="s">
+      <c r="A36" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B36" s="11" t="s">
+      <c r="B36" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C36" s="12" t="s">
+      <c r="C36" s="7" t="s">
         <v>82</v>
       </c>
-      <c r="D36" s="13" t="s">
+      <c r="D36" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="E36" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F36" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G36" s="13"/>
+      <c r="E36" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F36" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G36" s="8"/>
     </row>
     <row r="37" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="10" t="s">
+      <c r="A37" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B37" s="11" t="s">
+      <c r="B37" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C37" s="12" t="s">
+      <c r="C37" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="D37" s="13" t="s">
+      <c r="D37" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="E37" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F37" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G37" s="13"/>
+      <c r="E37" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F37" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G37" s="8"/>
     </row>
     <row r="38" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B38" s="11" t="s">
+      <c r="A38" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B38" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C38" s="12" t="s">
+      <c r="C38" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="D38" s="13" t="s">
+      <c r="D38" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="E38" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F38" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G38" s="13"/>
+      <c r="E38" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F38" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G38" s="8"/>
     </row>
     <row r="39" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="9" t="s">
+      <c r="A39" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="B39" s="20"/>
-      <c r="C39" s="20"/>
-      <c r="D39" s="20"/>
-      <c r="E39" s="20"/>
-      <c r="F39" s="20"/>
-      <c r="G39" s="20"/>
+      <c r="B39" s="15"/>
+      <c r="C39" s="15"/>
+      <c r="D39" s="15"/>
+      <c r="E39" s="15"/>
+      <c r="F39" s="15"/>
+      <c r="G39" s="15"/>
     </row>
     <row r="40" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B40" s="11" t="s">
+      <c r="A40" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B40" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C40" s="12" t="s">
+      <c r="C40" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="D40" s="13" t="s">
+      <c r="D40" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="E40" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F40" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G40" s="13"/>
+      <c r="E40" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F40" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G40" s="8"/>
     </row>
     <row r="41" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B41" s="11" t="s">
+      <c r="A41" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B41" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C41" s="12" t="s">
+      <c r="C41" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="D41" s="13" t="s">
+      <c r="D41" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="E41" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F41" s="14" t="s">
+      <c r="E41" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F41" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G41" s="13"/>
+      <c r="G41" s="8"/>
     </row>
     <row r="42" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A42" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B42" s="11" t="s">
+      <c r="A42" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B42" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C42" s="12" t="s">
+      <c r="C42" s="7" t="s">
         <v>93</v>
       </c>
-      <c r="D42" s="13" t="s">
+      <c r="D42" s="8" t="s">
         <v>94</v>
       </c>
-      <c r="E42" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F42" s="14" t="s">
+      <c r="E42" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F42" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G42" s="13"/>
+      <c r="G42" s="8"/>
     </row>
     <row r="43" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A43" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B43" s="18" t="s">
+      <c r="A43" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B43" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="C43" s="17" t="s">
+      <c r="C43" s="12" t="s">
         <v>95</v>
       </c>
-      <c r="D43" s="18" t="s">
+      <c r="D43" s="13" t="s">
         <v>96</v>
       </c>
-      <c r="E43" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="F43" s="19" t="s">
+      <c r="E43" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="F43" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="G43" s="18"/>
+      <c r="G43" s="13"/>
     </row>
     <row r="44" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B44" s="11" t="s">
+      <c r="A44" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B44" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C44" s="12" t="s">
+      <c r="C44" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="D44" s="13" t="s">
+      <c r="D44" s="8" t="s">
         <v>98</v>
       </c>
-      <c r="E44" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F44" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G44" s="13"/>
+      <c r="E44" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F44" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G44" s="8"/>
     </row>
     <row r="45" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B45" s="11" t="s">
+      <c r="A45" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B45" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C45" s="12" t="s">
+      <c r="C45" s="7" t="s">
         <v>99</v>
       </c>
-      <c r="D45" s="13" t="s">
+      <c r="D45" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="E45" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F45" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G45" s="13"/>
+      <c r="E45" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F45" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G45" s="8"/>
     </row>
     <row r="46" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B46" s="11" t="s">
+      <c r="A46" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B46" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C46" s="12" t="s">
+      <c r="C46" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="D46" s="13" t="s">
+      <c r="D46" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="E46" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F46" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G46" s="13"/>
+      <c r="E46" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F46" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G46" s="8"/>
     </row>
     <row r="47" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B47" s="11" t="s">
+      <c r="A47" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B47" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C47" s="12" t="s">
+      <c r="C47" s="7" t="s">
         <v>103</v>
       </c>
-      <c r="D47" s="13" t="s">
+      <c r="D47" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="E47" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F47" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G47" s="13"/>
+      <c r="E47" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F47" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G47" s="8"/>
     </row>
     <row r="48" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="9" t="s">
+      <c r="A48" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="B48" s="20"/>
-      <c r="C48" s="20"/>
-      <c r="D48" s="20"/>
-      <c r="E48" s="20"/>
-      <c r="F48" s="20"/>
-      <c r="G48" s="20"/>
+      <c r="B48" s="15"/>
+      <c r="C48" s="15"/>
+      <c r="D48" s="15"/>
+      <c r="E48" s="15"/>
+      <c r="F48" s="15"/>
+      <c r="G48" s="15"/>
     </row>
     <row r="49" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A49" s="10" t="s">
+      <c r="A49" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B49" s="18" t="s">
+      <c r="B49" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="C49" s="17" t="s">
+      <c r="C49" s="12" t="s">
         <v>106</v>
       </c>
-      <c r="D49" s="18" t="s">
+      <c r="D49" s="13" t="s">
         <v>107</v>
       </c>
-      <c r="E49" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="F49" s="19" t="s">
+      <c r="E49" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="F49" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="G49" s="18" t="s">
+      <c r="G49" s="13" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="50" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A50" s="10" t="s">
+      <c r="A50" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B50" s="11" t="s">
+      <c r="B50" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="C50" s="12" t="s">
+      <c r="C50" s="7" t="s">
         <v>109</v>
       </c>
-      <c r="D50" s="13" t="s">
+      <c r="D50" s="8" t="s">
         <v>110</v>
       </c>
-      <c r="E50" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F50" s="14" t="s">
+      <c r="E50" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F50" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="G50" s="13" t="s">
+      <c r="G50" s="8" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="51" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A51" s="10" t="s">
+      <c r="A51" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B51" s="11" t="s">
+      <c r="B51" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="C51" s="12" t="s">
+      <c r="C51" s="7" t="s">
         <v>112</v>
       </c>
-      <c r="D51" s="13" t="s">
+      <c r="D51" s="8" t="s">
         <v>113</v>
       </c>
-      <c r="E51" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F51" s="14" t="s">
+      <c r="E51" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F51" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="G51" s="13" t="s">
+      <c r="G51" s="8" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="52" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A52" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B52" s="11" t="s">
+      <c r="A52" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B52" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="C52" s="12" t="s">
+      <c r="C52" s="7" t="s">
         <v>115</v>
       </c>
-      <c r="D52" s="13" t="s">
+      <c r="D52" s="8" t="s">
         <v>116</v>
       </c>
-      <c r="E52" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F52" s="14" t="s">
+      <c r="E52" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F52" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="G52" s="13"/>
+      <c r="G52" s="8"/>
     </row>
     <row r="53" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A53" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B53" s="11" t="s">
+      <c r="A53" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B53" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="C53" s="12" t="s">
+      <c r="C53" s="7" t="s">
         <v>117</v>
       </c>
-      <c r="D53" s="13" t="s">
+      <c r="D53" s="8" t="s">
         <v>118</v>
       </c>
-      <c r="E53" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F53" s="14" t="s">
+      <c r="E53" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F53" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="G53" s="13"/>
+      <c r="G53" s="8"/>
     </row>
     <row r="54" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A54" s="17" t="s">
-        <v>59</v>
-      </c>
-      <c r="B54" s="18" t="s">
+      <c r="A54" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="B54" s="13" t="s">
         <v>119</v>
       </c>
-      <c r="C54" s="17" t="s">
+      <c r="C54" s="12" t="s">
         <v>120</v>
       </c>
-      <c r="D54" s="18" t="s">
+      <c r="D54" s="13" t="s">
         <v>121</v>
       </c>
-      <c r="E54" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="F54" s="19" t="s">
+      <c r="E54" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="F54" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="G54" s="18" t="s">
+      <c r="G54" s="13" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="55" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A55" s="9" t="s">
+      <c r="A55" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="B55" s="20"/>
-      <c r="C55" s="20"/>
-      <c r="D55" s="20"/>
-      <c r="E55" s="20"/>
-      <c r="F55" s="20"/>
-      <c r="G55" s="20"/>
+      <c r="B55" s="15"/>
+      <c r="C55" s="15"/>
+      <c r="D55" s="15"/>
+      <c r="E55" s="15"/>
+      <c r="F55" s="15"/>
+      <c r="G55" s="15"/>
     </row>
     <row r="56" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A56" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B56" s="11" t="s">
+      <c r="A56" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B56" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C56" s="12" t="s">
+      <c r="C56" s="7" t="s">
         <v>125</v>
       </c>
-      <c r="D56" s="13" t="s">
+      <c r="D56" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="E56" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F56" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G56" s="13"/>
+      <c r="E56" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F56" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G56" s="8"/>
     </row>
     <row r="57" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A57" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B57" s="11" t="s">
+      <c r="A57" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B57" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C57" s="12" t="s">
+      <c r="C57" s="7" t="s">
         <v>127</v>
       </c>
-      <c r="D57" s="13" t="s">
+      <c r="D57" s="8" t="s">
         <v>128</v>
       </c>
-      <c r="E57" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F57" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G57" s="13"/>
+      <c r="E57" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F57" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G57" s="8"/>
     </row>
     <row r="58" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A58" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B58" s="11" t="s">
+      <c r="A58" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B58" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C58" s="12" t="s">
+      <c r="C58" s="7" t="s">
         <v>129</v>
       </c>
-      <c r="D58" s="13" t="s">
+      <c r="D58" s="8" t="s">
         <v>130</v>
       </c>
-      <c r="E58" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F58" s="14" t="s">
+      <c r="E58" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F58" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G58" s="13"/>
+      <c r="G58" s="8"/>
     </row>
     <row r="59" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A59" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="B59" s="1"/>
-      <c r="C59" s="1"/>
-      <c r="D59" s="1"/>
-      <c r="E59" s="1"/>
-      <c r="F59" s="1"/>
-      <c r="G59" s="1"/>
+      <c r="A59" s="25" t="s">
+        <v>59</v>
+      </c>
+      <c r="B59" s="25"/>
+      <c r="C59" s="25"/>
+      <c r="D59" s="25"/>
+      <c r="E59" s="25"/>
+      <c r="F59" s="25"/>
+      <c r="G59" s="25"/>
     </row>
     <row r="60" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A60" s="9" t="s">
+      <c r="A60" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="B60" s="20"/>
-      <c r="C60" s="20"/>
-      <c r="D60" s="20"/>
-      <c r="E60" s="20"/>
-      <c r="F60" s="20"/>
-      <c r="G60" s="20"/>
+      <c r="B60" s="15"/>
+      <c r="C60" s="15"/>
+      <c r="D60" s="15"/>
+      <c r="E60" s="15"/>
+      <c r="F60" s="15"/>
+      <c r="G60" s="15"/>
     </row>
     <row r="61" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A61" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B61" s="11" t="s">
+      <c r="A61" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B61" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C61" s="12" t="s">
+      <c r="C61" s="7" t="s">
         <v>132</v>
       </c>
-      <c r="D61" s="13" t="s">
+      <c r="D61" s="8" t="s">
         <v>133</v>
       </c>
-      <c r="E61" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F61" s="14" t="s">
+      <c r="E61" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F61" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G61" s="13"/>
+      <c r="G61" s="8"/>
     </row>
     <row r="62" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A62" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B62" s="11" t="s">
+      <c r="A62" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B62" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C62" s="12" t="s">
+      <c r="C62" s="7" t="s">
         <v>134</v>
       </c>
-      <c r="D62" s="13" t="s">
+      <c r="D62" s="8" t="s">
         <v>135</v>
       </c>
-      <c r="E62" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F62" s="14" t="s">
+      <c r="E62" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F62" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G62" s="13"/>
+      <c r="G62" s="8"/>
     </row>
     <row r="63" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A63" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B63" s="11" t="s">
+      <c r="A63" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B63" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C63" s="12" t="s">
+      <c r="C63" s="7" t="s">
         <v>136</v>
       </c>
-      <c r="D63" s="13" t="s">
+      <c r="D63" s="8" t="s">
         <v>137</v>
       </c>
-      <c r="E63" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F63" s="14" t="s">
+      <c r="E63" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F63" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G63" s="13"/>
+      <c r="G63" s="8"/>
     </row>
     <row r="64" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A64" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="B64" s="1"/>
-      <c r="C64" s="1"/>
-      <c r="D64" s="1"/>
-      <c r="E64" s="1"/>
-      <c r="F64" s="1"/>
-      <c r="G64" s="1"/>
+      <c r="A64" s="25" t="s">
+        <v>59</v>
+      </c>
+      <c r="B64" s="25"/>
+      <c r="C64" s="25"/>
+      <c r="D64" s="25"/>
+      <c r="E64" s="25"/>
+      <c r="F64" s="25"/>
+      <c r="G64" s="25"/>
     </row>
     <row r="65" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A65" s="9" t="s">
+      <c r="A65" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="B65" s="20"/>
-      <c r="C65" s="20"/>
-      <c r="D65" s="20"/>
-      <c r="E65" s="20"/>
-      <c r="F65" s="20"/>
-      <c r="G65" s="20"/>
+      <c r="B65" s="15"/>
+      <c r="C65" s="15"/>
+      <c r="D65" s="15"/>
+      <c r="E65" s="15"/>
+      <c r="F65" s="15"/>
+      <c r="G65" s="15"/>
     </row>
     <row r="66" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A66" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B66" s="11" t="s">
+      <c r="A66" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B66" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C66" s="12" t="s">
+      <c r="C66" s="7" t="s">
         <v>139</v>
       </c>
-      <c r="D66" s="13" t="s">
+      <c r="D66" s="8" t="s">
         <v>140</v>
       </c>
-      <c r="E66" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F66" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G66" s="13"/>
+      <c r="E66" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F66" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G66" s="8"/>
     </row>
     <row r="67" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A67" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B67" s="11" t="s">
+      <c r="A67" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B67" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C67" s="12" t="s">
+      <c r="C67" s="7" t="s">
         <v>141</v>
       </c>
-      <c r="D67" s="13" t="s">
+      <c r="D67" s="8" t="s">
         <v>142</v>
       </c>
-      <c r="E67" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F67" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G67" s="13"/>
+      <c r="E67" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F67" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G67" s="8"/>
     </row>
     <row r="68" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A68" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B68" s="11" t="s">
+      <c r="A68" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B68" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C68" s="12" t="s">
+      <c r="C68" s="7" t="s">
         <v>143</v>
       </c>
-      <c r="D68" s="13" t="s">
+      <c r="D68" s="8" t="s">
         <v>144</v>
       </c>
-      <c r="E68" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F68" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G68" s="13"/>
+      <c r="E68" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F68" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G68" s="8"/>
     </row>
     <row r="69" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A69" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B69" s="11" t="s">
+      <c r="A69" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B69" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="C69" s="12" t="s">
+      <c r="C69" s="7" t="s">
         <v>145</v>
       </c>
-      <c r="D69" s="13" t="s">
+      <c r="D69" s="8" t="s">
         <v>146</v>
       </c>
-      <c r="E69" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F69" s="14" t="s">
+      <c r="E69" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F69" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G69" s="13"/>
+      <c r="G69" s="8"/>
     </row>
     <row r="70" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A70" s="9" t="s">
+      <c r="A70" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="B70" s="20"/>
-      <c r="C70" s="20"/>
-      <c r="D70" s="20"/>
-      <c r="E70" s="20"/>
-      <c r="F70" s="20"/>
-      <c r="G70" s="20"/>
+      <c r="B70" s="15"/>
+      <c r="C70" s="15"/>
+      <c r="D70" s="15"/>
+      <c r="E70" s="15"/>
+      <c r="F70" s="15"/>
+      <c r="G70" s="15"/>
     </row>
     <row r="71" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A71" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B71" s="11" t="s">
+      <c r="A71" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B71" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C71" s="12" t="s">
+      <c r="C71" s="7" t="s">
         <v>148</v>
       </c>
-      <c r="D71" s="13" t="s">
+      <c r="D71" s="8" t="s">
         <v>149</v>
       </c>
-      <c r="E71" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F71" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G71" s="13" t="s">
+      <c r="E71" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F71" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G71" s="8" t="s">
         <v>150</v>
       </c>
     </row>
     <row r="72" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A72" s="17" t="s">
-        <v>59</v>
-      </c>
-      <c r="B72" s="18" t="s">
+      <c r="A72" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="B72" s="13" t="s">
         <v>63</v>
       </c>
-      <c r="C72" s="17" t="s">
+      <c r="C72" s="12" t="s">
         <v>151</v>
       </c>
-      <c r="D72" s="18" t="s">
+      <c r="D72" s="13" t="s">
         <v>152</v>
       </c>
-      <c r="E72" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="F72" s="19" t="s">
+      <c r="E72" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="F72" s="14" t="s">
         <v>66</v>
       </c>
-      <c r="G72" s="18" t="s">
+      <c r="G72" s="13" t="s">
         <v>153</v>
       </c>
     </row>
     <row r="73" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A73" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B73" s="11" t="s">
+      <c r="A73" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B73" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C73" s="12" t="s">
+      <c r="C73" s="7" t="s">
         <v>154</v>
       </c>
-      <c r="D73" s="13" t="s">
+      <c r="D73" s="8" t="s">
         <v>155</v>
       </c>
-      <c r="E73" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F73" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G73" s="13"/>
+      <c r="E73" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F73" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G73" s="8"/>
     </row>
     <row r="74" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A74" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B74" s="11" t="s">
+      <c r="A74" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B74" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C74" s="12" t="s">
+      <c r="C74" s="7" t="s">
         <v>156</v>
       </c>
-      <c r="D74" s="13" t="s">
+      <c r="D74" s="8" t="s">
         <v>157</v>
       </c>
-      <c r="E74" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F74" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G74" s="13"/>
+      <c r="E74" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F74" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G74" s="8"/>
     </row>
     <row r="75" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A75" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B75" s="11" t="s">
+      <c r="A75" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B75" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="C75" s="12" t="s">
+      <c r="C75" s="7" t="s">
         <v>158</v>
       </c>
-      <c r="D75" s="13" t="s">
+      <c r="D75" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="E75" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F75" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G75" s="13"/>
+      <c r="E75" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F75" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G75" s="8"/>
     </row>
     <row r="76" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A76" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B76" s="18" t="s">
+      <c r="A76" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B76" s="13" t="s">
         <v>29</v>
       </c>
-      <c r="C76" s="17" t="s">
+      <c r="C76" s="12" t="s">
         <v>160</v>
       </c>
-      <c r="D76" s="18" t="s">
+      <c r="D76" s="13" t="s">
         <v>161</v>
       </c>
-      <c r="E76" s="18" t="s">
-        <v>15</v>
-      </c>
-      <c r="F76" s="21" t="s">
-        <v>16</v>
-      </c>
-      <c r="G76" s="18"/>
+      <c r="E76" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="F76" s="16" t="s">
+        <v>16</v>
+      </c>
+      <c r="G76" s="13"/>
     </row>
     <row r="77" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A77" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B77" s="11" t="s">
+      <c r="A77" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B77" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C77" s="12" t="s">
+      <c r="C77" s="7" t="s">
         <v>162</v>
       </c>
-      <c r="D77" s="13" t="s">
+      <c r="D77" s="8" t="s">
         <v>163</v>
       </c>
-      <c r="E77" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F77" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G77" s="13"/>
+      <c r="E77" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F77" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G77" s="8"/>
     </row>
     <row r="78" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A78" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B78" s="11" t="s">
+      <c r="A78" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B78" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C78" s="12" t="s">
+      <c r="C78" s="7" t="s">
         <v>164</v>
       </c>
-      <c r="D78" s="13" t="s">
+      <c r="D78" s="8" t="s">
         <v>165</v>
       </c>
-      <c r="E78" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F78" s="14" t="s">
+      <c r="E78" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F78" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G78" s="13"/>
+      <c r="G78" s="8"/>
     </row>
     <row r="79" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A79" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B79" s="11" t="s">
+      <c r="A79" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B79" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C79" s="12" t="s">
+      <c r="C79" s="7" t="s">
         <v>166</v>
       </c>
-      <c r="D79" s="13" t="s">
+      <c r="D79" s="8" t="s">
         <v>167</v>
       </c>
-      <c r="E79" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F79" s="14" t="s">
+      <c r="E79" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F79" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G79" s="13"/>
+      <c r="G79" s="8"/>
     </row>
     <row r="80" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A80" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B80" s="11" t="s">
+      <c r="A80" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B80" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="C80" s="12" t="s">
+      <c r="C80" s="7" t="s">
         <v>168</v>
       </c>
-      <c r="D80" s="13" t="s">
+      <c r="D80" s="8" t="s">
         <v>169</v>
       </c>
-      <c r="E80" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F80" s="14" t="s">
+      <c r="E80" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F80" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G80" s="13"/>
+      <c r="G80" s="8"/>
     </row>
     <row r="81" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A81" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B81" s="11" t="s">
+      <c r="A81" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B81" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="C81" s="12" t="s">
+      <c r="C81" s="7" t="s">
         <v>170</v>
       </c>
-      <c r="D81" s="13" t="s">
+      <c r="D81" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="E81" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F81" s="14" t="s">
+      <c r="E81" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F81" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G81" s="13"/>
+      <c r="G81" s="8"/>
     </row>
     <row r="82" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A82" s="9" t="s">
+      <c r="A82" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="B82" s="20"/>
-      <c r="C82" s="20"/>
-      <c r="D82" s="20"/>
-      <c r="E82" s="20"/>
-      <c r="F82" s="20"/>
-      <c r="G82" s="20"/>
+      <c r="B82" s="15"/>
+      <c r="C82" s="15"/>
+      <c r="D82" s="15"/>
+      <c r="E82" s="15"/>
+      <c r="F82" s="15"/>
+      <c r="G82" s="15"/>
     </row>
     <row r="83" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A83" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B83" s="11" t="s">
+      <c r="A83" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B83" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C83" s="12" t="s">
+      <c r="C83" s="7" t="s">
         <v>173</v>
       </c>
-      <c r="D83" s="13" t="s">
+      <c r="D83" s="8" t="s">
         <v>174</v>
       </c>
-      <c r="E83" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F83" s="14" t="s">
+      <c r="E83" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F83" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G83" s="13"/>
+      <c r="G83" s="8"/>
     </row>
     <row r="84" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A84" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B84" s="11" t="s">
+      <c r="A84" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B84" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C84" s="12" t="s">
+      <c r="C84" s="7" t="s">
         <v>175</v>
       </c>
-      <c r="D84" s="13" t="s">
+      <c r="D84" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="E84" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F84" s="14" t="s">
+      <c r="E84" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F84" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="G84" s="13"/>
+      <c r="G84" s="8"/>
     </row>
     <row r="85" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A85" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B85" s="11" t="s">
+      <c r="A85" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B85" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="C85" s="12" t="s">
+      <c r="C85" s="7" t="s">
         <v>177</v>
       </c>
-      <c r="D85" s="13" t="s">
+      <c r="D85" s="8" t="s">
         <v>178</v>
       </c>
-      <c r="E85" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F85" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G85" s="13"/>
+      <c r="E85" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F85" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G85" s="8"/>
     </row>
     <row r="86" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A86" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B86" s="11" t="s">
+      <c r="A86" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B86" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="C86" s="12" t="s">
+      <c r="C86" s="7" t="s">
         <v>179</v>
       </c>
-      <c r="D86" s="13" t="s">
+      <c r="D86" s="8" t="s">
         <v>180</v>
       </c>
-      <c r="E86" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F86" s="14" t="s">
+      <c r="E86" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F86" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="G86" s="13"/>
+      <c r="G86" s="8"/>
     </row>
     <row r="87" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A87" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="B87" s="11" t="s">
+      <c r="A87" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B87" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="C87" s="12" t="s">
+      <c r="C87" s="7" t="s">
         <v>181</v>
       </c>
-      <c r="D87" s="13" t="s">
+      <c r="D87" s="8" t="s">
         <v>182</v>
       </c>
-      <c r="E87" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F87" s="14" t="s">
+      <c r="E87" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="F87" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="G87" s="13"/>
+      <c r="G87" s="8"/>
     </row>
     <row r="88" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A88" s="22"/>
-      <c r="B88" s="22"/>
-      <c r="C88" s="22"/>
-      <c r="D88" s="22"/>
-      <c r="E88" s="22"/>
-      <c r="F88" s="22"/>
-      <c r="G88" s="22"/>
+      <c r="A88" s="17"/>
+      <c r="B88" s="17"/>
+      <c r="C88" s="17"/>
+      <c r="D88" s="17"/>
+      <c r="E88" s="17"/>
+      <c r="F88" s="17"/>
+      <c r="G88" s="17"/>
     </row>
     <row r="89" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A89" s="22"/>
-      <c r="B89" s="22"/>
-      <c r="C89" s="22"/>
-      <c r="D89" s="22"/>
-      <c r="E89" s="22"/>
-      <c r="F89" s="22"/>
-      <c r="G89" s="22"/>
+      <c r="A89" s="17"/>
+      <c r="B89" s="17"/>
+      <c r="C89" s="17"/>
+      <c r="D89" s="17"/>
+      <c r="E89" s="17"/>
+      <c r="F89" s="17"/>
+      <c r="G89" s="17"/>
     </row>
     <row r="90" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A90" s="22"/>
-      <c r="B90" s="22"/>
-      <c r="C90" s="22"/>
-      <c r="D90" s="22"/>
-      <c r="E90" s="22"/>
-      <c r="F90" s="22"/>
-      <c r="G90" s="22"/>
+      <c r="A90" s="17"/>
+      <c r="B90" s="17"/>
+      <c r="C90" s="17"/>
+      <c r="D90" s="17"/>
+      <c r="E90" s="17"/>
+      <c r="F90" s="17"/>
+      <c r="G90" s="17"/>
     </row>
     <row r="91" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A91" s="22"/>
-      <c r="B91" s="22"/>
-      <c r="C91" s="22"/>
-      <c r="D91" s="22"/>
-      <c r="E91" s="22"/>
-      <c r="F91" s="22"/>
-      <c r="G91" s="22"/>
+      <c r="A91" s="17"/>
+      <c r="B91" s="17"/>
+      <c r="C91" s="17"/>
+      <c r="D91" s="17"/>
+      <c r="E91" s="17"/>
+      <c r="F91" s="17"/>
+      <c r="G91" s="17"/>
     </row>
     <row r="92" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A92" s="22"/>
-      <c r="B92" s="22"/>
-      <c r="C92" s="22"/>
-      <c r="D92" s="22"/>
-      <c r="E92" s="22"/>
-      <c r="F92" s="22"/>
-      <c r="G92" s="22"/>
+      <c r="A92" s="17"/>
+      <c r="B92" s="17"/>
+      <c r="C92" s="17"/>
+      <c r="D92" s="17"/>
+      <c r="E92" s="17"/>
+      <c r="F92" s="17"/>
+      <c r="G92" s="17"/>
     </row>
     <row r="93" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A93" s="22"/>
-      <c r="B93" s="22"/>
-      <c r="C93" s="22"/>
-      <c r="D93" s="22"/>
-      <c r="E93" s="22"/>
-      <c r="F93" s="22"/>
-      <c r="G93" s="22"/>
+      <c r="A93" s="17"/>
+      <c r="B93" s="17"/>
+      <c r="C93" s="17"/>
+      <c r="D93" s="17"/>
+      <c r="E93" s="17"/>
+      <c r="F93" s="17"/>
+      <c r="G93" s="17"/>
     </row>
     <row r="94" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A94" s="22"/>
-      <c r="B94" s="22"/>
-      <c r="C94" s="22"/>
-      <c r="D94" s="22"/>
-      <c r="E94" s="22"/>
-      <c r="F94" s="22"/>
-      <c r="G94" s="22"/>
+      <c r="A94" s="17"/>
+      <c r="B94" s="17"/>
+      <c r="C94" s="17"/>
+      <c r="D94" s="17"/>
+      <c r="E94" s="17"/>
+      <c r="F94" s="17"/>
+      <c r="G94" s="17"/>
     </row>
     <row r="95" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A95" s="22"/>
-      <c r="B95" s="22"/>
-      <c r="C95" s="22"/>
-      <c r="D95" s="22"/>
-      <c r="E95" s="22"/>
-      <c r="F95" s="22"/>
-      <c r="G95" s="22"/>
+      <c r="A95" s="17"/>
+      <c r="B95" s="17"/>
+      <c r="C95" s="17"/>
+      <c r="D95" s="17"/>
+      <c r="E95" s="17"/>
+      <c r="F95" s="17"/>
+      <c r="G95" s="17"/>
     </row>
     <row r="96" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A96" s="22"/>
-      <c r="B96" s="22"/>
-      <c r="C96" s="22"/>
-      <c r="D96" s="22"/>
-      <c r="E96" s="22"/>
-      <c r="F96" s="22"/>
-      <c r="G96" s="22"/>
+      <c r="A96" s="17"/>
+      <c r="B96" s="17"/>
+      <c r="C96" s="17"/>
+      <c r="D96" s="17"/>
+      <c r="E96" s="17"/>
+      <c r="F96" s="17"/>
+      <c r="G96" s="17"/>
     </row>
     <row r="97" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A97" s="22"/>
-      <c r="B97" s="22"/>
-      <c r="C97" s="22"/>
-      <c r="D97" s="22"/>
-      <c r="E97" s="22"/>
-      <c r="F97" s="22"/>
-      <c r="G97" s="22"/>
+      <c r="A97" s="17"/>
+      <c r="B97" s="17"/>
+      <c r="C97" s="17"/>
+      <c r="D97" s="17"/>
+      <c r="E97" s="17"/>
+      <c r="F97" s="17"/>
+      <c r="G97" s="17"/>
     </row>
     <row r="98" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A98" s="22"/>
-      <c r="B98" s="22"/>
-      <c r="C98" s="22"/>
-      <c r="D98" s="22"/>
-      <c r="E98" s="22"/>
-      <c r="F98" s="22"/>
-      <c r="G98" s="22"/>
+      <c r="A98" s="17"/>
+      <c r="B98" s="17"/>
+      <c r="C98" s="17"/>
+      <c r="D98" s="17"/>
+      <c r="E98" s="17"/>
+      <c r="F98" s="17"/>
+      <c r="G98" s="17"/>
     </row>
     <row r="99" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A99" s="22"/>
-      <c r="B99" s="22"/>
-      <c r="C99" s="22"/>
-      <c r="D99" s="22"/>
-      <c r="E99" s="22"/>
-      <c r="F99" s="22"/>
-      <c r="G99" s="22"/>
+      <c r="A99" s="17"/>
+      <c r="B99" s="17"/>
+      <c r="C99" s="17"/>
+      <c r="D99" s="17"/>
+      <c r="E99" s="17"/>
+      <c r="F99" s="17"/>
+      <c r="G99" s="17"/>
     </row>
     <row r="100" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A100" s="22"/>
-      <c r="B100" s="22"/>
-      <c r="C100" s="22"/>
-      <c r="D100" s="22"/>
-      <c r="E100" s="22"/>
-      <c r="F100" s="22"/>
-      <c r="G100" s="22"/>
+      <c r="A100" s="17"/>
+      <c r="B100" s="17"/>
+      <c r="C100" s="17"/>
+      <c r="D100" s="17"/>
+      <c r="E100" s="17"/>
+      <c r="F100" s="17"/>
+      <c r="G100" s="17"/>
     </row>
     <row r="101" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A101" s="22"/>
-      <c r="B101" s="22"/>
-      <c r="C101" s="22"/>
-      <c r="D101" s="22"/>
-      <c r="E101" s="22"/>
-      <c r="F101" s="22"/>
-      <c r="G101" s="22"/>
+      <c r="A101" s="17"/>
+      <c r="B101" s="17"/>
+      <c r="C101" s="17"/>
+      <c r="D101" s="17"/>
+      <c r="E101" s="17"/>
+      <c r="F101" s="17"/>
+      <c r="G101" s="17"/>
     </row>
     <row r="102" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A102" s="22"/>
-      <c r="B102" s="22"/>
-      <c r="C102" s="22"/>
-      <c r="D102" s="22"/>
-      <c r="E102" s="22"/>
-      <c r="F102" s="22"/>
-      <c r="G102" s="22"/>
+      <c r="A102" s="17"/>
+      <c r="B102" s="17"/>
+      <c r="C102" s="17"/>
+      <c r="D102" s="17"/>
+      <c r="E102" s="17"/>
+      <c r="F102" s="17"/>
+      <c r="G102" s="17"/>
     </row>
     <row r="103" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A103" s="22"/>
-      <c r="B103" s="22"/>
-      <c r="C103" s="22"/>
-      <c r="D103" s="22"/>
-      <c r="E103" s="22"/>
-      <c r="F103" s="22"/>
-      <c r="G103" s="22"/>
+      <c r="A103" s="17"/>
+      <c r="B103" s="17"/>
+      <c r="C103" s="17"/>
+      <c r="D103" s="17"/>
+      <c r="E103" s="17"/>
+      <c r="F103" s="17"/>
+      <c r="G103" s="17"/>
     </row>
     <row r="104" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A104" s="22"/>
-      <c r="B104" s="22"/>
-      <c r="C104" s="22"/>
-      <c r="D104" s="22"/>
-      <c r="E104" s="22"/>
-      <c r="F104" s="22"/>
-      <c r="G104" s="22"/>
+      <c r="A104" s="17"/>
+      <c r="B104" s="17"/>
+      <c r="C104" s="17"/>
+      <c r="D104" s="17"/>
+      <c r="E104" s="17"/>
+      <c r="F104" s="17"/>
+      <c r="G104" s="17"/>
     </row>
     <row r="105" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A105" s="22"/>
-      <c r="B105" s="22"/>
-      <c r="C105" s="22"/>
-      <c r="D105" s="22"/>
-      <c r="E105" s="22"/>
-      <c r="F105" s="22"/>
-      <c r="G105" s="22"/>
+      <c r="A105" s="17"/>
+      <c r="B105" s="17"/>
+      <c r="C105" s="17"/>
+      <c r="D105" s="17"/>
+      <c r="E105" s="17"/>
+      <c r="F105" s="17"/>
+      <c r="G105" s="17"/>
     </row>
     <row r="106" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A106" s="22"/>
-      <c r="B106" s="22"/>
-      <c r="C106" s="22"/>
-      <c r="D106" s="22"/>
-      <c r="E106" s="22"/>
-      <c r="F106" s="22"/>
-      <c r="G106" s="22"/>
+      <c r="A106" s="17"/>
+      <c r="B106" s="17"/>
+      <c r="C106" s="17"/>
+      <c r="D106" s="17"/>
+      <c r="E106" s="17"/>
+      <c r="F106" s="17"/>
+      <c r="G106" s="17"/>
     </row>
     <row r="107" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A107" s="22"/>
-      <c r="B107" s="22"/>
-      <c r="C107" s="22"/>
-      <c r="D107" s="22"/>
-      <c r="E107" s="22"/>
-      <c r="F107" s="22"/>
-      <c r="G107" s="22"/>
+      <c r="A107" s="17"/>
+      <c r="B107" s="17"/>
+      <c r="C107" s="17"/>
+      <c r="D107" s="17"/>
+      <c r="E107" s="17"/>
+      <c r="F107" s="17"/>
+      <c r="G107" s="17"/>
     </row>
     <row r="108" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A108" s="22"/>
-      <c r="B108" s="22"/>
-      <c r="C108" s="22"/>
-      <c r="D108" s="22"/>
-      <c r="E108" s="22"/>
-      <c r="F108" s="22"/>
-      <c r="G108" s="22"/>
+      <c r="A108" s="17"/>
+      <c r="B108" s="17"/>
+      <c r="C108" s="17"/>
+      <c r="D108" s="17"/>
+      <c r="E108" s="17"/>
+      <c r="F108" s="17"/>
+      <c r="G108" s="17"/>
     </row>
     <row r="109" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A109" s="22"/>
-      <c r="B109" s="22"/>
-      <c r="C109" s="22"/>
-      <c r="D109" s="22"/>
-      <c r="E109" s="22"/>
-      <c r="F109" s="22"/>
-      <c r="G109" s="22"/>
+      <c r="A109" s="17"/>
+      <c r="B109" s="17"/>
+      <c r="C109" s="17"/>
+      <c r="D109" s="17"/>
+      <c r="E109" s="17"/>
+      <c r="F109" s="17"/>
+      <c r="G109" s="17"/>
     </row>
     <row r="110" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A110" s="22"/>
-      <c r="B110" s="22"/>
-      <c r="C110" s="22"/>
-      <c r="D110" s="22"/>
-      <c r="E110" s="22"/>
-      <c r="F110" s="22"/>
-      <c r="G110" s="22"/>
+      <c r="A110" s="17"/>
+      <c r="B110" s="17"/>
+      <c r="C110" s="17"/>
+      <c r="D110" s="17"/>
+      <c r="E110" s="17"/>
+      <c r="F110" s="17"/>
+      <c r="G110" s="17"/>
     </row>
     <row r="111" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A111" s="22"/>
-      <c r="B111" s="22"/>
-      <c r="C111" s="22"/>
-      <c r="D111" s="22"/>
-      <c r="E111" s="22"/>
-      <c r="F111" s="22"/>
-      <c r="G111" s="22"/>
+      <c r="A111" s="17"/>
+      <c r="B111" s="17"/>
+      <c r="C111" s="17"/>
+      <c r="D111" s="17"/>
+      <c r="E111" s="17"/>
+      <c r="F111" s="17"/>
+      <c r="G111" s="17"/>
     </row>
     <row r="112" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A112" s="22"/>
-      <c r="B112" s="22"/>
-      <c r="C112" s="22"/>
-      <c r="D112" s="22"/>
-      <c r="E112" s="22"/>
-      <c r="F112" s="22"/>
-      <c r="G112" s="22"/>
+      <c r="A112" s="17"/>
+      <c r="B112" s="17"/>
+      <c r="C112" s="17"/>
+      <c r="D112" s="17"/>
+      <c r="E112" s="17"/>
+      <c r="F112" s="17"/>
+      <c r="G112" s="17"/>
     </row>
     <row r="113" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A113" s="22"/>
-      <c r="B113" s="22"/>
-      <c r="C113" s="22"/>
-      <c r="D113" s="22"/>
-      <c r="E113" s="22"/>
-      <c r="F113" s="22"/>
-      <c r="G113" s="22"/>
+      <c r="A113" s="17"/>
+      <c r="B113" s="17"/>
+      <c r="C113" s="17"/>
+      <c r="D113" s="17"/>
+      <c r="E113" s="17"/>
+      <c r="F113" s="17"/>
+      <c r="G113" s="17"/>
     </row>
     <row r="114" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A114" s="22"/>
-      <c r="B114" s="22"/>
-      <c r="C114" s="22"/>
-      <c r="D114" s="22"/>
-      <c r="E114" s="22"/>
-      <c r="F114" s="22"/>
-      <c r="G114" s="22"/>
+      <c r="A114" s="17"/>
+      <c r="B114" s="17"/>
+      <c r="C114" s="17"/>
+      <c r="D114" s="17"/>
+      <c r="E114" s="17"/>
+      <c r="F114" s="17"/>
+      <c r="G114" s="17"/>
     </row>
     <row r="115" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A115" s="22"/>
-      <c r="B115" s="22"/>
-      <c r="C115" s="22"/>
-      <c r="D115" s="22"/>
-      <c r="E115" s="22"/>
-      <c r="F115" s="22"/>
-      <c r="G115" s="22"/>
+      <c r="A115" s="17"/>
+      <c r="B115" s="17"/>
+      <c r="C115" s="17"/>
+      <c r="D115" s="17"/>
+      <c r="E115" s="17"/>
+      <c r="F115" s="17"/>
+      <c r="G115" s="17"/>
     </row>
     <row r="116" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A116" s="22"/>
-      <c r="B116" s="22"/>
-      <c r="C116" s="22"/>
-      <c r="D116" s="22"/>
-      <c r="E116" s="22"/>
-      <c r="F116" s="22"/>
-      <c r="G116" s="22"/>
+      <c r="A116" s="17"/>
+      <c r="B116" s="17"/>
+      <c r="C116" s="17"/>
+      <c r="D116" s="17"/>
+      <c r="E116" s="17"/>
+      <c r="F116" s="17"/>
+      <c r="G116" s="17"/>
     </row>
     <row r="117" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A117" s="22"/>
-      <c r="B117" s="22"/>
-      <c r="C117" s="22"/>
-      <c r="D117" s="22"/>
-      <c r="E117" s="22"/>
-      <c r="F117" s="22"/>
-      <c r="G117" s="22"/>
+      <c r="A117" s="17"/>
+      <c r="B117" s="17"/>
+      <c r="C117" s="17"/>
+      <c r="D117" s="17"/>
+      <c r="E117" s="17"/>
+      <c r="F117" s="17"/>
+      <c r="G117" s="17"/>
     </row>
     <row r="118" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A118" s="22"/>
-      <c r="B118" s="22"/>
-      <c r="C118" s="22"/>
-      <c r="D118" s="22"/>
-      <c r="E118" s="22"/>
-      <c r="F118" s="22"/>
-      <c r="G118" s="22"/>
+      <c r="A118" s="17"/>
+      <c r="B118" s="17"/>
+      <c r="C118" s="17"/>
+      <c r="D118" s="17"/>
+      <c r="E118" s="17"/>
+      <c r="F118" s="17"/>
+      <c r="G118" s="17"/>
     </row>
     <row r="119" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A119" s="22"/>
-      <c r="B119" s="22"/>
-      <c r="C119" s="22"/>
-      <c r="D119" s="22"/>
-      <c r="E119" s="22"/>
-      <c r="F119" s="22"/>
-      <c r="G119" s="22"/>
+      <c r="A119" s="17"/>
+      <c r="B119" s="17"/>
+      <c r="C119" s="17"/>
+      <c r="D119" s="17"/>
+      <c r="E119" s="17"/>
+      <c r="F119" s="17"/>
+      <c r="G119" s="17"/>
     </row>
     <row r="120" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A120" s="22"/>
-      <c r="B120" s="22"/>
-      <c r="C120" s="22"/>
-      <c r="D120" s="22"/>
-      <c r="E120" s="22"/>
-      <c r="F120" s="22"/>
-      <c r="G120" s="22"/>
+      <c r="A120" s="17"/>
+      <c r="B120" s="17"/>
+      <c r="C120" s="17"/>
+      <c r="D120" s="17"/>
+      <c r="E120" s="17"/>
+      <c r="F120" s="17"/>
+      <c r="G120" s="17"/>
     </row>
     <row r="121" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A121" s="22"/>
-      <c r="B121" s="22"/>
-      <c r="C121" s="22"/>
-      <c r="D121" s="22"/>
-      <c r="E121" s="22"/>
-      <c r="F121" s="22"/>
-      <c r="G121" s="22"/>
+      <c r="A121" s="17"/>
+      <c r="B121" s="17"/>
+      <c r="C121" s="17"/>
+      <c r="D121" s="17"/>
+      <c r="E121" s="17"/>
+      <c r="F121" s="17"/>
+      <c r="G121" s="17"/>
     </row>
     <row r="122" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A122" s="22"/>
-      <c r="B122" s="22"/>
-      <c r="C122" s="22"/>
-      <c r="D122" s="22"/>
-      <c r="E122" s="22"/>
-      <c r="F122" s="22"/>
-      <c r="G122" s="22"/>
+      <c r="A122" s="17"/>
+      <c r="B122" s="17"/>
+      <c r="C122" s="17"/>
+      <c r="D122" s="17"/>
+      <c r="E122" s="17"/>
+      <c r="F122" s="17"/>
+      <c r="G122" s="17"/>
     </row>
     <row r="123" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A123" s="22"/>
-      <c r="B123" s="22"/>
-      <c r="C123" s="22"/>
-      <c r="D123" s="22"/>
-      <c r="E123" s="22"/>
-      <c r="F123" s="22"/>
-      <c r="G123" s="22"/>
+      <c r="A123" s="17"/>
+      <c r="B123" s="17"/>
+      <c r="C123" s="17"/>
+      <c r="D123" s="17"/>
+      <c r="E123" s="17"/>
+      <c r="F123" s="17"/>
+      <c r="G123" s="17"/>
     </row>
     <row r="124" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A124" s="22"/>
-      <c r="B124" s="22"/>
-      <c r="C124" s="22"/>
-      <c r="D124" s="22"/>
-      <c r="E124" s="22"/>
-      <c r="F124" s="22"/>
-      <c r="G124" s="22"/>
+      <c r="A124" s="17"/>
+      <c r="B124" s="17"/>
+      <c r="C124" s="17"/>
+      <c r="D124" s="17"/>
+      <c r="E124" s="17"/>
+      <c r="F124" s="17"/>
+      <c r="G124" s="17"/>
     </row>
     <row r="125" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A125" s="22"/>
-      <c r="B125" s="22"/>
-      <c r="C125" s="22"/>
-      <c r="D125" s="22"/>
-      <c r="E125" s="22"/>
-      <c r="F125" s="22"/>
-      <c r="G125" s="22"/>
+      <c r="A125" s="17"/>
+      <c r="B125" s="17"/>
+      <c r="C125" s="17"/>
+      <c r="D125" s="17"/>
+      <c r="E125" s="17"/>
+      <c r="F125" s="17"/>
+      <c r="G125" s="17"/>
     </row>
     <row r="126" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A126" s="22"/>
-      <c r="B126" s="22"/>
-      <c r="C126" s="22"/>
-      <c r="D126" s="22"/>
-      <c r="E126" s="22"/>
-      <c r="F126" s="22"/>
-      <c r="G126" s="22"/>
+      <c r="A126" s="17"/>
+      <c r="B126" s="17"/>
+      <c r="C126" s="17"/>
+      <c r="D126" s="17"/>
+      <c r="E126" s="17"/>
+      <c r="F126" s="17"/>
+      <c r="G126" s="17"/>
     </row>
   </sheetData>
   <autoFilter ref="A4:G80" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
@@ -3205,7 +3205,7 @@
     <mergeCell ref="A10:G10"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" error="Choisir: ✅ ⬜ ⏳ ❌" prompt="✅=Fait ⬜=À faire ⏳=En cours ❌=Bloqué" sqref="A6:A9 A11:A17 A19:A23 A25:A29 A31:A33 A35:A42 A44:A48 A50:A53 A55:A58 A60:A63 A65:A74 A76:A80" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" error="Choisir: ✅ ⬜ ⏳ ❌" prompt="✅=Fait ⬜=À faire ⏳=En cours ❌=Bloqué" sqref="A6:A9 A11:A17 A19:A23 A25:A33 A35:A42 A44:A48 A50:A53 A55:A58 A60:A63 A65:A74 A76:A80" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"✅,⬜,⏳,❌"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -3235,331 +3235,331 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="26" t="s">
         <v>183</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
+      <c r="B1" s="26"/>
+      <c r="C1" s="26"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="26"/>
     </row>
     <row r="2" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="18" t="s">
         <v>184</v>
       </c>
-      <c r="B2" s="23" t="s">
+      <c r="B2" s="18" t="s">
         <v>185</v>
       </c>
-      <c r="C2" s="23" t="s">
+      <c r="C2" s="18" t="s">
         <v>186</v>
       </c>
-      <c r="D2" s="23" t="s">
+      <c r="D2" s="18" t="s">
         <v>187</v>
       </c>
-      <c r="E2" s="23" t="s">
+      <c r="E2" s="18" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="24" t="s">
+      <c r="A3" s="19" t="s">
         <v>189</v>
       </c>
-      <c r="B3" s="25">
+      <c r="B3" s="20">
         <f>COUNTIF('Checklist Production'!A6:A9,"✅")</f>
         <v>4</v>
       </c>
-      <c r="C3" s="10">
+      <c r="C3" s="1">
         <f>COUNTIF('Checklist Production'!A6:A9,"⬜")</f>
         <v>0</v>
       </c>
-      <c r="D3" s="14">
+      <c r="D3" s="9">
         <f>COUNTIF('Checklist Production'!A6:A9,"⏳")</f>
         <v>0</v>
       </c>
-      <c r="E3" s="26">
+      <c r="E3" s="21">
         <f>COUNTIF('Checklist Production'!A6:A9,"❌")</f>
         <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="24" t="s">
+      <c r="A4" s="19" t="s">
         <v>190</v>
       </c>
-      <c r="B4" s="25">
+      <c r="B4" s="20">
         <f>COUNTIF('Checklist Production'!A11:A17,"✅")</f>
         <v>7</v>
       </c>
-      <c r="C4" s="10">
+      <c r="C4" s="1">
         <f>COUNTIF('Checklist Production'!A11:A17,"⬜")</f>
         <v>0</v>
       </c>
-      <c r="D4" s="14">
+      <c r="D4" s="9">
         <f>COUNTIF('Checklist Production'!A11:A17,"⏳")</f>
         <v>0</v>
       </c>
-      <c r="E4" s="26">
+      <c r="E4" s="21">
         <f>COUNTIF('Checklist Production'!A11:A17,"❌")</f>
         <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A5" s="24" t="s">
+      <c r="A5" s="19" t="s">
         <v>191</v>
       </c>
-      <c r="B5" s="25">
+      <c r="B5" s="20">
         <f>COUNTIF('Checklist Production'!A19:A23,"✅")</f>
         <v>4</v>
       </c>
-      <c r="C5" s="10">
+      <c r="C5" s="1">
         <f>COUNTIF('Checklist Production'!A19:A23,"⬜")</f>
         <v>0</v>
       </c>
-      <c r="D5" s="14">
+      <c r="D5" s="9">
         <f>COUNTIF('Checklist Production'!A19:A23,"⏳")</f>
         <v>0</v>
       </c>
-      <c r="E5" s="26">
+      <c r="E5" s="21">
         <f>COUNTIF('Checklist Production'!A19:A23,"❌")</f>
         <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="24" t="s">
+      <c r="A6" s="19" t="s">
         <v>192</v>
       </c>
-      <c r="B6" s="25">
+      <c r="B6" s="20">
         <f>COUNTIF('Checklist Production'!A25:A29,"✅")</f>
         <v>3</v>
       </c>
-      <c r="C6" s="10">
+      <c r="C6" s="1">
         <f>COUNTIF('Checklist Production'!A25:A29,"⬜")</f>
         <v>1</v>
       </c>
-      <c r="D6" s="14">
+      <c r="D6" s="9">
         <f>COUNTIF('Checklist Production'!A25:A29,"⏳")</f>
         <v>0</v>
       </c>
-      <c r="E6" s="26">
+      <c r="E6" s="21">
         <f>COUNTIF('Checklist Production'!A25:A29,"❌")</f>
         <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="24" t="s">
+      <c r="A7" s="19" t="s">
         <v>193</v>
       </c>
-      <c r="B7" s="25">
+      <c r="B7" s="20">
         <f>COUNTIF('Checklist Production'!A31:A33,"✅")</f>
         <v>0</v>
       </c>
-      <c r="C7" s="10">
+      <c r="C7" s="1">
         <f>COUNTIF('Checklist Production'!A31:A33,"⬜")</f>
         <v>3</v>
       </c>
-      <c r="D7" s="14">
+      <c r="D7" s="9">
         <f>COUNTIF('Checklist Production'!A31:A33,"⏳")</f>
         <v>0</v>
       </c>
-      <c r="E7" s="26">
+      <c r="E7" s="21">
         <f>COUNTIF('Checklist Production'!A31:A33,"❌")</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="24" t="s">
+      <c r="A8" s="19" t="s">
         <v>194</v>
       </c>
-      <c r="B8" s="25">
+      <c r="B8" s="20">
         <f>COUNTIF('Checklist Production'!A35:A42,"✅")</f>
-        <v>2</v>
-      </c>
-      <c r="C8" s="10">
+        <v>3</v>
+      </c>
+      <c r="C8" s="1">
         <f>COUNTIF('Checklist Production'!A35:A42,"⬜")</f>
-        <v>4</v>
-      </c>
-      <c r="D8" s="14">
+        <v>3</v>
+      </c>
+      <c r="D8" s="9">
         <f>COUNTIF('Checklist Production'!A35:A42,"⏳")</f>
         <v>0</v>
       </c>
-      <c r="E8" s="26">
+      <c r="E8" s="21">
         <f>COUNTIF('Checklist Production'!A35:A42,"❌")</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="24" t="s">
+      <c r="A9" s="19" t="s">
         <v>195</v>
       </c>
-      <c r="B9" s="25">
+      <c r="B9" s="20">
         <f>COUNTIF('Checklist Production'!A44:A48,"✅")</f>
         <v>0</v>
       </c>
-      <c r="C9" s="10">
+      <c r="C9" s="1">
         <f>COUNTIF('Checklist Production'!A44:A48,"⬜")</f>
         <v>4</v>
       </c>
-      <c r="D9" s="14">
+      <c r="D9" s="9">
         <f>COUNTIF('Checklist Production'!A44:A48,"⏳")</f>
         <v>0</v>
       </c>
-      <c r="E9" s="26">
+      <c r="E9" s="21">
         <f>COUNTIF('Checklist Production'!A44:A48,"❌")</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="24" t="s">
+      <c r="A10" s="19" t="s">
         <v>196</v>
       </c>
-      <c r="B10" s="25">
+      <c r="B10" s="20">
         <f>COUNTIF('Checklist Production'!A50:A53,"✅")</f>
         <v>2</v>
       </c>
-      <c r="C10" s="10">
+      <c r="C10" s="1">
         <f>COUNTIF('Checklist Production'!A50:A53,"⬜")</f>
         <v>2</v>
       </c>
-      <c r="D10" s="14">
+      <c r="D10" s="9">
         <f>COUNTIF('Checklist Production'!A50:A53,"⏳")</f>
         <v>0</v>
       </c>
-      <c r="E10" s="26">
+      <c r="E10" s="21">
         <f>COUNTIF('Checklist Production'!A50:A53,"❌")</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="24" t="s">
+      <c r="A11" s="19" t="s">
         <v>197</v>
       </c>
-      <c r="B11" s="25">
+      <c r="B11" s="20">
         <f>COUNTIF('Checklist Production'!A55:A58,"✅")</f>
         <v>0</v>
       </c>
-      <c r="C11" s="10">
+      <c r="C11" s="1">
         <f>COUNTIF('Checklist Production'!A55:A58,"⬜")</f>
         <v>3</v>
       </c>
-      <c r="D11" s="14">
+      <c r="D11" s="9">
         <f>COUNTIF('Checklist Production'!A55:A58,"⏳")</f>
         <v>0</v>
       </c>
-      <c r="E11" s="26">
+      <c r="E11" s="21">
         <f>COUNTIF('Checklist Production'!A55:A58,"❌")</f>
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="24" t="s">
+      <c r="A12" s="19" t="s">
         <v>198</v>
       </c>
-      <c r="B12" s="25">
+      <c r="B12" s="20">
         <f>COUNTIF('Checklist Production'!A60:A63,"✅")</f>
         <v>0</v>
       </c>
-      <c r="C12" s="10">
+      <c r="C12" s="1">
         <f>COUNTIF('Checklist Production'!A60:A63,"⬜")</f>
         <v>3</v>
       </c>
-      <c r="D12" s="14">
+      <c r="D12" s="9">
         <f>COUNTIF('Checklist Production'!A60:A63,"⏳")</f>
         <v>0</v>
       </c>
-      <c r="E12" s="26">
+      <c r="E12" s="21">
         <f>COUNTIF('Checklist Production'!A60:A63,"❌")</f>
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="24" t="s">
+      <c r="A13" s="19" t="s">
         <v>199</v>
       </c>
-      <c r="B13" s="25">
+      <c r="B13" s="20">
         <f>COUNTIF('Checklist Production'!A65:A74,"✅")</f>
         <v>0</v>
       </c>
-      <c r="C13" s="10">
+      <c r="C13" s="1">
         <f>COUNTIF('Checklist Production'!A65:A74,"⬜")</f>
         <v>8</v>
       </c>
-      <c r="D13" s="14">
+      <c r="D13" s="9">
         <f>COUNTIF('Checklist Production'!A65:A74,"⏳")</f>
         <v>0</v>
       </c>
-      <c r="E13" s="26">
+      <c r="E13" s="21">
         <f>COUNTIF('Checklist Production'!A65:A74,"❌")</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="24" t="s">
+      <c r="A14" s="19" t="s">
         <v>200</v>
       </c>
-      <c r="B14" s="25">
+      <c r="B14" s="20">
         <f>COUNTIF('Checklist Production'!A76:A80,"✅")</f>
         <v>0</v>
       </c>
-      <c r="C14" s="10">
+      <c r="C14" s="1">
         <f>COUNTIF('Checklist Production'!A76:A80,"⬜")</f>
         <v>5</v>
       </c>
-      <c r="D14" s="14">
+      <c r="D14" s="9">
         <f>COUNTIF('Checklist Production'!A76:A80,"⏳")</f>
         <v>0</v>
       </c>
-      <c r="E14" s="26">
+      <c r="E14" s="21">
         <f>COUNTIF('Checklist Production'!A76:A80,"❌")</f>
         <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="27" t="s">
+      <c r="A15" s="22" t="s">
         <v>201</v>
       </c>
-      <c r="B15" s="28">
+      <c r="B15" s="23">
         <f>SUM(B3:B14)</f>
-        <v>22</v>
-      </c>
-      <c r="C15" s="28">
+        <v>23</v>
+      </c>
+      <c r="C15" s="23">
         <f>SUM(C3:C14)</f>
-        <v>33</v>
-      </c>
-      <c r="D15" s="28">
+        <v>32</v>
+      </c>
+      <c r="D15" s="23">
         <f>SUM(D3:D14)</f>
         <v>0</v>
       </c>
-      <c r="E15" s="28">
+      <c r="E15" s="23">
         <f>SUM(E3:E14)</f>
         <v>2</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="22"/>
-      <c r="B16" s="22"/>
-      <c r="C16" s="22"/>
-      <c r="D16" s="22"/>
-      <c r="E16" s="22"/>
+      <c r="A16" s="17"/>
+      <c r="B16" s="17"/>
+      <c r="C16" s="17"/>
+      <c r="D16" s="17"/>
+      <c r="E16" s="17"/>
     </row>
     <row r="17" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="22"/>
-      <c r="B17" s="22"/>
-      <c r="C17" s="22"/>
-      <c r="D17" s="22"/>
-      <c r="E17" s="22"/>
+      <c r="A17" s="17"/>
+      <c r="B17" s="17"/>
+      <c r="C17" s="17"/>
+      <c r="D17" s="17"/>
+      <c r="E17" s="17"/>
     </row>
     <row r="18" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A18" s="22"/>
-      <c r="B18" s="22"/>
-      <c r="C18" s="22"/>
-      <c r="D18" s="22"/>
-      <c r="E18" s="22"/>
+      <c r="A18" s="17"/>
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="17"/>
     </row>
     <row r="19" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="22"/>
-      <c r="B19" s="22"/>
-      <c r="C19" s="22"/>
-      <c r="D19" s="22"/>
-      <c r="E19" s="22"/>
+      <c r="A19" s="17"/>
+      <c r="B19" s="17"/>
+      <c r="C19" s="17"/>
+      <c r="D19" s="17"/>
+      <c r="E19" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>